<commit_message>
Add Savings, Investments, and Circles as separate money-location screens with shared create and move actions.
</commit_message>
<xml_diff>
--- a/public/templates/fintrack-transactions-import-template.xlsx
+++ b/public/templates/fintrack-transactions-import-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MyPortfolioProjects\fintrack-app\fintrack-fe\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258B5A5E-6E96-4CBC-8A40-805C1D62B896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41B6A28-4699-4F0C-9309-C8F9E0A88582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A57337A4-A16A-457D-ABB2-C6993C0A5F73}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A57337A4-A16A-457D-ABB2-C6993C0A5F73}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>currency (optional)</t>
-  </si>
-  <si>
-    <t>description (optional)</t>
   </si>
   <si>
     <t>income</t>
@@ -94,6 +91,9 @@
   </si>
   <si>
     <t>Freelance invoice</t>
+  </si>
+  <si>
+    <t>note (optional)</t>
   </si>
 </sst>
 </file>
@@ -507,7 +507,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -534,20 +534,20 @@
         <v>46235</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="3">
         <v>85000</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -574,22 +574,22 @@
         <v>46238</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="E3" s="3">
         <v>500</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -616,20 +616,20 @@
         <v>46239</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="3">
         <v>120</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -656,13 +656,13 @@
         <v>46240</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" s="3">
         <v>3200</v>
@@ -694,20 +694,20 @@
         <v>46241</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="3">
         <v>1899</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -734,20 +734,20 @@
         <v>46242</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="3">
         <v>12000</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>

</xml_diff>